<commit_message>
fix(data): aggregate historical municipal components
</commit_message>
<xml_diff>
--- a/docs/Raw Data/Municipalities/geostat-population-regional-gdp/municipal-population-and-regional-gdp.xlsx
+++ b/docs/Raw Data/Municipalities/geostat-population-regional-gdp/municipal-population-and-regional-gdp.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R4dea224f262d4e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Population" sheetId="2" r:id="Rfb111adcceaf435e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional GDP" sheetId="3" r:id="R1355dd1b93cb41aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geography map" sheetId="4" r:id="R23710fb2f1d040af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R84a1de35e4f64689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Population" sheetId="2" r:id="R561c4d48166648ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional GDP" sheetId="3" r:id="Ra52c7e161c6c4890"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geography map" sheetId="4" r:id="R93cd7c6c3efa4fa1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -361,7 +361,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="88" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -397,67 +397,75 @@
         <x:v>2015–2025; 704 rows; 0 official gaps.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str">
-        <x:v>Regional GDP definition</x:v>
+        <x:v>Population component rules</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>Total GDP by region at current prices in million GEL; not municipal GDP.</x:v>
+        <x:v>7 explicit sum rules; 21 municipality-year rows in 2015–2017 add separately published starred city cells to the surrounding municipality.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str">
-        <x:v>Regional GDP coverage</x:v>
+        <x:v>Regional GDP definition</x:v>
       </x:c>
       <x:c r="B7" s="21" t="str">
-        <x:v>2010–2024; 165 rows; 0 official gaps.</x:v>
+        <x:v>Total GDP by region at current prices in million GEL; not municipal GDP.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str">
-        <x:v>Validation status</x:v>
+        <x:v>Regional GDP coverage</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>complete</x:v>
+        <x:v>2010–2024; 165 rows; 0 official gaps.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="20" t="str">
-        <x:v>Estimates created</x:v>
-      </x:c>
-      <x:c r="B9" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>Validation status</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>complete</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="20" t="str">
-        <x:v>Retrieval/review date</x:v>
-      </x:c>
-      <x:c r="B10" s="24" t="n">
-        <x:v>46237</x:v>
+        <x:v>Estimates created</x:v>
+      </x:c>
+      <x:c r="B10" s="21" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="20" t="str">
-        <x:v>Population source page</x:v>
-      </x:c>
-      <x:c r="B11" s="21" t="str">
-        <x:v>https://www.geostat.ge/en/modules/categories/41/population</x:v>
+        <x:v>Retrieval/review date</x:v>
+      </x:c>
+      <x:c r="B11" s="24" t="n">
+        <x:v>46237</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="20" t="str">
+        <x:v>Population source page</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>https://www.geostat.ge/en/modules/categories/41/population</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="20" t="str">
         <x:v>Regional GDP source page</x:v>
       </x:c>
-      <x:c r="B12" s="21" t="str">
+      <x:c r="B13" s="21" t="str">
         <x:v>https://www.geostat.ge/en/modules/categories/23/gross-domestic-product-gdp</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="22" t="str">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="22" t="str">
         <x:v>Exclusions</x:v>
       </x:c>
-      <x:c r="B13" s="23" t="str">
+      <x:c r="B14" s="23" t="str">
         <x:v>Codes 05, 42, 43, 46, and 64; national GDP total retained only for reconciliation.</x:v>
       </x:c>
     </x:row>
@@ -483,7 +491,7 @@
     <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="116" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="122" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -919,10 +927,10 @@
         <x:v>region.kakheti</x:v>
       </x:c>
       <x:c r="E12" s="30" t="n">
-        <x:v>38.4</x:v>
+        <x:v>58.2</x:v>
       </x:c>
       <x:c r="F12" s="31" t="n">
-        <x:v>38400</x:v>
+        <x:v>58200</x:v>
       </x:c>
       <x:c r="G12" s="32" t="n">
         <x:v>42005</x:v>
@@ -937,7 +945,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>Source sheet "1"; source row 39; year 2015 column W (cell W39); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 39 + 35; year 2015 column W (cells W39 + W35); population_thousand = W39 + W35; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L12" s="32" t="n">
         <x:v>46237</x:v>
@@ -1603,10 +1611,10 @@
         <x:v>region.samegrelo_zemo_svaneti</x:v>
       </x:c>
       <x:c r="E30" s="30" t="n">
-        <x:v>62.9</x:v>
+        <x:v>106.7</x:v>
       </x:c>
       <x:c r="F30" s="31" t="n">
-        <x:v>62900</x:v>
+        <x:v>106700</x:v>
       </x:c>
       <x:c r="G30" s="32" t="n">
         <x:v>42005</x:v>
@@ -1621,7 +1629,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K30" t="str">
-        <x:v>Source sheet "1"; source row 61; year 2015 column W (cell W61); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 61 + 58; year 2015 column W (cells W61 + W58); population_thousand = W61 + W58; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L30" s="32" t="n">
         <x:v>46237</x:v>
@@ -1907,10 +1915,10 @@
         <x:v>region.shida_kartli</x:v>
       </x:c>
       <x:c r="E38" s="30" t="n">
-        <x:v>77.6</x:v>
+        <x:v>125.4</x:v>
       </x:c>
       <x:c r="F38" s="31" t="n">
-        <x:v>77600</x:v>
+        <x:v>125400</x:v>
       </x:c>
       <x:c r="G38" s="32" t="n">
         <x:v>42005</x:v>
@@ -1925,7 +1933,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K38" t="str">
-        <x:v>Source sheet "1"; source row 86; year 2015 column W (cell W86); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 86 + 85; year 2015 column W (cells W86 + W85); population_thousand = W86 + W85; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L38" s="32" t="n">
         <x:v>46237</x:v>
@@ -2363,10 +2371,10 @@
         <x:v>region.guria</x:v>
       </x:c>
       <x:c r="E50" s="30" t="n">
-        <x:v>47.8</x:v>
+        <x:v>62.8</x:v>
       </x:c>
       <x:c r="F50" s="31" t="n">
-        <x:v>47800</x:v>
+        <x:v>62800</x:v>
       </x:c>
       <x:c r="G50" s="32" t="n">
         <x:v>42005</x:v>
@@ -2381,7 +2389,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K50" t="str">
-        <x:v>Source sheet "1"; source row 19; year 2015 column W (cell W19); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 19 + 17; year 2015 column W (cells W19 + W17); population_thousand = W19 + W17; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L50" s="32" t="n">
         <x:v>46237</x:v>
@@ -2591,10 +2599,10 @@
         <x:v>region.samtskhe_javakheti</x:v>
       </x:c>
       <x:c r="E56" s="30" t="n">
-        <x:v>22.9</x:v>
+        <x:v>39.2</x:v>
       </x:c>
       <x:c r="F56" s="31" t="n">
-        <x:v>22900</x:v>
+        <x:v>39200</x:v>
       </x:c>
       <x:c r="G56" s="32" t="n">
         <x:v>42005</x:v>
@@ -2609,7 +2617,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K56" t="str">
-        <x:v>Source sheet "1"; source row 73; year 2015 column W (cell W73); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 73 + 69; year 2015 column W (cells W73 + W69); population_thousand = W73 + W69; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L56" s="32" t="n">
         <x:v>46237</x:v>
@@ -2743,10 +2751,10 @@
         <x:v>region.mtskheta_mtianeti</x:v>
       </x:c>
       <x:c r="E60" s="30" t="n">
-        <x:v>46.8</x:v>
+        <x:v>54.6</x:v>
       </x:c>
       <x:c r="F60" s="31" t="n">
-        <x:v>46800</x:v>
+        <x:v>54600</x:v>
       </x:c>
       <x:c r="G60" s="32" t="n">
         <x:v>42005</x:v>
@@ -2761,7 +2769,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K60" t="str">
-        <x:v>Source sheet "1"; source row 49; year 2015 column W (cell W49); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 49 + 45; year 2015 column W (cells W49 + W45); population_thousand = W49 + W45; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L60" s="32" t="n">
         <x:v>46237</x:v>
@@ -2819,10 +2827,10 @@
         <x:v>region.racha_lechkhumi_kvemo_svaneti</x:v>
       </x:c>
       <x:c r="E62" s="30" t="n">
-        <x:v>9.1</x:v>
+        <x:v>11.2</x:v>
       </x:c>
       <x:c r="F62" s="31" t="n">
-        <x:v>9100</x:v>
+        <x:v>11200</x:v>
       </x:c>
       <x:c r="G62" s="32" t="n">
         <x:v>42005</x:v>
@@ -2837,7 +2845,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K62" t="str">
-        <x:v>Source sheet "1"; source row 53; year 2015 column W (cell W53); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 53 + 52; year 2015 column W (cells W53 + W52); population_thousand = W53 + W52; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L62" s="32" t="n">
         <x:v>46237</x:v>
@@ -3351,10 +3359,10 @@
         <x:v>region.kakheti</x:v>
       </x:c>
       <x:c r="E76" s="30" t="n">
-        <x:v>37.9</x:v>
+        <x:v>57.7</x:v>
       </x:c>
       <x:c r="F76" s="31" t="n">
-        <x:v>37900</x:v>
+        <x:v>57700</x:v>
       </x:c>
       <x:c r="G76" s="32" t="n">
         <x:v>42370</x:v>
@@ -3369,7 +3377,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K76" t="str">
-        <x:v>Source sheet "1"; source row 39; year 2016 column X (cell X39); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 39 + 35; year 2016 column X (cells X39 + X35); population_thousand = X39 + X35; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L76" s="32" t="n">
         <x:v>46237</x:v>
@@ -4035,10 +4043,10 @@
         <x:v>region.samegrelo_zemo_svaneti</x:v>
       </x:c>
       <x:c r="E94" s="30" t="n">
-        <x:v>62.3</x:v>
+        <x:v>105.7</x:v>
       </x:c>
       <x:c r="F94" s="31" t="n">
-        <x:v>62300</x:v>
+        <x:v>105700</x:v>
       </x:c>
       <x:c r="G94" s="32" t="n">
         <x:v>42370</x:v>
@@ -4053,7 +4061,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K94" t="str">
-        <x:v>Source sheet "1"; source row 61; year 2016 column X (cell X61); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 61 + 58; year 2016 column X (cells X61 + X58); population_thousand = X61 + X58; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L94" s="32" t="n">
         <x:v>46237</x:v>
@@ -4339,10 +4347,10 @@
         <x:v>region.shida_kartli</x:v>
       </x:c>
       <x:c r="E102" s="30" t="n">
-        <x:v>77.3</x:v>
+        <x:v>124.7</x:v>
       </x:c>
       <x:c r="F102" s="31" t="n">
-        <x:v>77300</x:v>
+        <x:v>124700</x:v>
       </x:c>
       <x:c r="G102" s="32" t="n">
         <x:v>42370</x:v>
@@ -4357,7 +4365,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K102" t="str">
-        <x:v>Source sheet "1"; source row 86; year 2016 column X (cell X86); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 86 + 85; year 2016 column X (cells X86 + X85); population_thousand = X86 + X85; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L102" s="32" t="n">
         <x:v>46237</x:v>
@@ -4795,10 +4803,10 @@
         <x:v>region.guria</x:v>
       </x:c>
       <x:c r="E114" s="30" t="n">
-        <x:v>47.4</x:v>
+        <x:v>62.3</x:v>
       </x:c>
       <x:c r="F114" s="31" t="n">
-        <x:v>47400</x:v>
+        <x:v>62300</x:v>
       </x:c>
       <x:c r="G114" s="32" t="n">
         <x:v>42370</x:v>
@@ -4813,7 +4821,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K114" t="str">
-        <x:v>Source sheet "1"; source row 19; year 2016 column X (cell X19); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 19 + 17; year 2016 column X (cells X19 + X17); population_thousand = X19 + X17; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L114" s="32" t="n">
         <x:v>46237</x:v>
@@ -5023,10 +5031,10 @@
         <x:v>region.samtskhe_javakheti</x:v>
       </x:c>
       <x:c r="E120" s="30" t="n">
-        <x:v>22.8</x:v>
+        <x:v>39.2</x:v>
       </x:c>
       <x:c r="F120" s="31" t="n">
-        <x:v>22800</x:v>
+        <x:v>39200</x:v>
       </x:c>
       <x:c r="G120" s="32" t="n">
         <x:v>42370</x:v>
@@ -5041,7 +5049,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K120" t="str">
-        <x:v>Source sheet "1"; source row 73; year 2016 column X (cell X73); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 73 + 69; year 2016 column X (cells X73 + X69); population_thousand = X73 + X69; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L120" s="32" t="n">
         <x:v>46237</x:v>
@@ -5175,10 +5183,10 @@
         <x:v>region.mtskheta_mtianeti</x:v>
       </x:c>
       <x:c r="E124" s="30" t="n">
-        <x:v>46.7</x:v>
+        <x:v>54.4</x:v>
       </x:c>
       <x:c r="F124" s="31" t="n">
-        <x:v>46700</x:v>
+        <x:v>54400</x:v>
       </x:c>
       <x:c r="G124" s="32" t="n">
         <x:v>42370</x:v>
@@ -5193,7 +5201,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K124" t="str">
-        <x:v>Source sheet "1"; source row 49; year 2016 column X (cell X49); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 49 + 45; year 2016 column X (cells X49 + X45); population_thousand = X49 + X45; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L124" s="32" t="n">
         <x:v>46237</x:v>
@@ -5251,10 +5259,10 @@
         <x:v>region.racha_lechkhumi_kvemo_svaneti</x:v>
       </x:c>
       <x:c r="E126" s="30" t="n">
-        <x:v>9</x:v>
+        <x:v>11.1</x:v>
       </x:c>
       <x:c r="F126" s="31" t="n">
-        <x:v>9000</x:v>
+        <x:v>11100</x:v>
       </x:c>
       <x:c r="G126" s="32" t="n">
         <x:v>42370</x:v>
@@ -5269,7 +5277,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K126" t="str">
-        <x:v>Source sheet "1"; source row 53; year 2016 column X (cell X53); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 53 + 52; year 2016 column X (cells X53 + X52); population_thousand = X53 + X52; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L126" s="32" t="n">
         <x:v>46237</x:v>
@@ -5783,10 +5791,10 @@
         <x:v>region.kakheti</x:v>
       </x:c>
       <x:c r="E140" s="30" t="n">
-        <x:v>37.4</x:v>
+        <x:v>57.2</x:v>
       </x:c>
       <x:c r="F140" s="31" t="n">
-        <x:v>37400</x:v>
+        <x:v>57200</x:v>
       </x:c>
       <x:c r="G140" s="32" t="n">
         <x:v>42736</x:v>
@@ -5801,7 +5809,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K140" t="str">
-        <x:v>Source sheet "1"; source row 39; year 2017 column Y (cell Y39); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 39 + 35; year 2017 column Y (cells Y39 + Y35); population_thousand = Y39 + Y35; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L140" s="32" t="n">
         <x:v>46237</x:v>
@@ -6467,10 +6475,10 @@
         <x:v>region.samegrelo_zemo_svaneti</x:v>
       </x:c>
       <x:c r="E158" s="30" t="n">
-        <x:v>61.5</x:v>
+        <x:v>104.2</x:v>
       </x:c>
       <x:c r="F158" s="31" t="n">
-        <x:v>61500</x:v>
+        <x:v>104200</x:v>
       </x:c>
       <x:c r="G158" s="32" t="n">
         <x:v>42736</x:v>
@@ -6485,7 +6493,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K158" t="str">
-        <x:v>Source sheet "1"; source row 61; year 2017 column Y (cell Y61); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 61 + 58; year 2017 column Y (cells Y61 + Y58); population_thousand = Y61 + Y58; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L158" s="32" t="n">
         <x:v>46237</x:v>
@@ -6771,10 +6779,10 @@
         <x:v>region.shida_kartli</x:v>
       </x:c>
       <x:c r="E166" s="30" t="n">
-        <x:v>76.9</x:v>
+        <x:v>123.8</x:v>
       </x:c>
       <x:c r="F166" s="31" t="n">
-        <x:v>76900</x:v>
+        <x:v>123800</x:v>
       </x:c>
       <x:c r="G166" s="32" t="n">
         <x:v>42736</x:v>
@@ -6789,7 +6797,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K166" t="str">
-        <x:v>Source sheet "1"; source row 86; year 2017 column Y (cell Y86); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 86 + 85; year 2017 column Y (cells Y86 + Y85); population_thousand = Y86 + Y85; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L166" s="32" t="n">
         <x:v>46237</x:v>
@@ -7227,10 +7235,10 @@
         <x:v>region.guria</x:v>
       </x:c>
       <x:c r="E178" s="30" t="n">
-        <x:v>47</x:v>
+        <x:v>61.8</x:v>
       </x:c>
       <x:c r="F178" s="31" t="n">
-        <x:v>47000</x:v>
+        <x:v>61800</x:v>
       </x:c>
       <x:c r="G178" s="32" t="n">
         <x:v>42736</x:v>
@@ -7245,7 +7253,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K178" t="str">
-        <x:v>Source sheet "1"; source row 19; year 2017 column Y (cell Y19); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 19 + 17; year 2017 column Y (cells Y19 + Y17); population_thousand = Y19 + Y17; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L178" s="32" t="n">
         <x:v>46237</x:v>
@@ -7455,10 +7463,10 @@
         <x:v>region.samtskhe_javakheti</x:v>
       </x:c>
       <x:c r="E184" s="30" t="n">
-        <x:v>22.7</x:v>
+        <x:v>39.3</x:v>
       </x:c>
       <x:c r="F184" s="31" t="n">
-        <x:v>22700</x:v>
+        <x:v>39300</x:v>
       </x:c>
       <x:c r="G184" s="32" t="n">
         <x:v>42736</x:v>
@@ -7473,7 +7481,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K184" t="str">
-        <x:v>Source sheet "1"; source row 73; year 2017 column Y (cell Y73); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 73 + 69; year 2017 column Y (cells Y73 + Y69); population_thousand = Y73 + Y69; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L184" s="32" t="n">
         <x:v>46237</x:v>
@@ -7607,10 +7615,10 @@
         <x:v>region.mtskheta_mtianeti</x:v>
       </x:c>
       <x:c r="E188" s="30" t="n">
-        <x:v>46.5</x:v>
+        <x:v>54.2</x:v>
       </x:c>
       <x:c r="F188" s="31" t="n">
-        <x:v>46500</x:v>
+        <x:v>54200</x:v>
       </x:c>
       <x:c r="G188" s="32" t="n">
         <x:v>42736</x:v>
@@ -7625,7 +7633,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K188" t="str">
-        <x:v>Source sheet "1"; source row 49; year 2017 column Y (cell Y49); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 49 + 45; year 2017 column Y (cells Y49 + Y45); population_thousand = Y49 + Y45; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L188" s="32" t="n">
         <x:v>46237</x:v>
@@ -7683,10 +7691,10 @@
         <x:v>region.racha_lechkhumi_kvemo_svaneti</x:v>
       </x:c>
       <x:c r="E190" s="30" t="n">
-        <x:v>8.8</x:v>
+        <x:v>10.8</x:v>
       </x:c>
       <x:c r="F190" s="31" t="n">
-        <x:v>8800</x:v>
+        <x:v>10800</x:v>
       </x:c>
       <x:c r="G190" s="32" t="n">
         <x:v>42736</x:v>
@@ -7701,7 +7709,7 @@
         <x:v>(thousands)</x:v>
       </x:c>
       <x:c r="K190" t="str">
-        <x:v>Source sheet "1"; source row 53; year 2017 column Y (cell Y53); retained published thousands; persons = thousands * 1000; no estimates.</x:v>
+        <x:v>Source sheet "1"; source rows 53 + 52; year 2017 column Y (cells Y53 + Y52); population_thousand = Y53 + Y52; persons = thousands * 1000; no estimates.</x:v>
       </x:c>
       <x:c r="L190" s="32" t="n">
         <x:v>46237</x:v>

</xml_diff>